<commit_message>
Fix: Sincronización de archivos y estructura
</commit_message>
<xml_diff>
--- a/casas.xlsx
+++ b/casas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10402"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fernandoperezescalante/real-estate-catalog/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hans_\OneDrive\Escritorio\Projectos\Real State\gestioninmobiliargalindo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84ADAE5F-FFC5-E248-8ED8-6B0431794C7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47D3990E-72F2-46CA-8BAD-C7684670B99B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="500" windowWidth="51200" windowHeight="27020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="28800" windowHeight="15285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template Excel para Script Pyth" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="83">
   <si>
     <t>id</t>
   </si>
@@ -138,12 +138,305 @@
   <si>
     <t>Disponible</t>
   </si>
+  <si>
+    <t>T-001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TERRENO </t>
+  </si>
+  <si>
+    <t xml:space="preserve">VENTA </t>
+  </si>
+  <si>
+    <t>1,050,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EL HAYA </t>
+  </si>
+  <si>
+    <t>Xalapa</t>
+  </si>
+  <si>
+    <t>330.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UBICADO EN EL HAYA 
+TERRENO  330 M2
+CUENTA CON ESCRITURA PUBLICA 
+TOMA DE AGUA
+</t>
+  </si>
+  <si>
+    <t>C-004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CASA </t>
+  </si>
+  <si>
+    <t xml:space="preserve">CASA HABITACION </t>
+  </si>
+  <si>
+    <t>2,100,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JARDINES </t>
+  </si>
+  <si>
+    <t>XALAPA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESTRENE COMODA CASA DE TRES RECAMARAS, JARDIN Y COCHERA, UBICADA A UNAS CUADRAS DE CAMINO ANTIGUO A NAOLINCO.
+105 M2 DE TERRENO.
+158 M2 DE CONSTRUCCION.
+INVERSION FIJA DE  $ 2, 100,000
+PLANTA BAJA:
+COCHERA PARA UN AUTO 
+1/2 BAÑO.
+SALA-COMEDOR.
+COCINA CON BARRA DESAYUNADOR.
+JARDIN.
+PLANTA ALTA:
+DOS RECAMARAS SECUNDARIAS.
+1 BAÑO COMPLETO COMPARTIDO.
+AMPLIA RECAMARA PRINCIPAL CON BAÑO COMPLETO.
+AZOTEA:
+AREA DE LAVADO TECHADA.
+</t>
+  </si>
+  <si>
+    <t>D-001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DEPRTANTO </t>
+  </si>
+  <si>
+    <t xml:space="preserve">DEPRTAMENTO ZONA JARDINES </t>
+  </si>
+  <si>
+    <t>VENTA</t>
+  </si>
+  <si>
+    <t>DEPARTAMENTO</t>
+  </si>
+  <si>
+    <t>1,550,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DEPARTAMENTOS  UBICADOS AUN COSTADO DE PLAZA CRISTAL 
+                                   $ 1,550,000
+Cajón de estacionamiento p/1 auto (la cochera es techada y con portón eléctrico).
+Cisterna.
+Sala-Comedor.
+Cocina integral con pequeña barra desayunador y gabinete de madera.
+Dos recámaras con clóset c/u. La principal cuenta con pequeño balcón.
+1 Baño completo.
+AZOTEA:
+Área de lavado y tendido.
+</t>
+  </si>
+  <si>
+    <t>C-005</t>
+  </si>
+  <si>
+    <t>3,000,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRANCAS </t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMILIANO ZAPATA </t>
+  </si>
+  <si>
+    <t xml:space="preserve">PLANTA BAJA:
+Cochera Techada p/3 autos.
+Cisterna de 10,000 LTS.
+Acceso independiente al patio trasero con pequeño jardín.
+Sala.
+Comedor con acceso al patio.
+Amplia Cocina con acceso al corredor.
+1 Recamara individual.
+1/2 Baño.
+                  PLANTA ALTA:
+Área de estudio.
+Amplia sala de TV.
+Área de juegos.
+Amplia recamara principal con baño completo, vestidor y balcón.
+Otras 2 recamaras secundarias con closet c/u.
+1 baño completo.
+Balcón trasero.
+                     AZOTEA:
+Área de lavado techado.
+Amplio ROFF GARDEN.
+</t>
+  </si>
+  <si>
+    <t>C-006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RESIDENCIAL LIRIOS </t>
+  </si>
+  <si>
+    <t>2,500,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COATEPEC </t>
+  </si>
+  <si>
+    <t xml:space="preserve">XALAPA </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> FRACCIONAMIENTO PRIVADO; CARRETERA LAS TRANCAS
+105 M2 DE TERRENO.
+146 M2 DE CONSTRUCCION.
+PLANTA BAJA:
+Cochera p/1 auto..
+Sala.
+1/2 Baño.
+Comedor.
+Cocina Integral.
+Área de lavado techado. 
+1 Recamara con closet y baño completo.
+PLANTA ALTA:
+Sala de T.V.
+Recamara principal con baño completo y vestidor.
+Recamara secundaria con closet, baño completo y balcón.
+</t>
+  </si>
+  <si>
+    <t>C-007</t>
+  </si>
+  <si>
+    <t>2,240,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PLANTA BAJA:
+Amplia cochera p/2 autos.
+1 Baño de visitas.
+Sala 
+Comedor.
+Cocina con barra desayunador.
+1 Recamara con closet y baño completo.
+PLANTA ALTA:
+Amplia recámara principal con baño completo y espacio de vestidor.
+Recamara secundaria con espacio de closet. 
+1 baño completo 
+Área de servicio y terraza.
+</t>
+  </si>
+  <si>
+    <t>C-008</t>
+  </si>
+  <si>
+    <t>CASARESIDENCIAL</t>
+  </si>
+  <si>
+    <t>3,190,000</t>
+  </si>
+  <si>
+    <t>MORADA DEL QUETZAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PLANTA BAJA:
+DOBLE COCHERA.
+CISTERNA DE 8,500 LTS
+1/2 BAÑO.
+SALA-COMEDOR.
+COCINA INTEGRAL Y CON ISLA CENTRAL.
+COLINDA CON AREA VERDE EN LA PARTE DE ATRAS.
+PLANTA ALTA:
+DOS RECAMARAS FRONTALES CON BALCON Y CLOSET C/U.
+1 BAÑO COMPLETO COMPARTIDO.
+AMPLIA RECAMARA PRINCIPAL CON VESTIDOR Y BAÑO COMPLETO.
+AZOTEA:
+AREA DE LAVADO TECHADO.
+AREA EMPERGOLADA.
+BARRA CON TARJA Y ASADOR.
+ROFF GARDEN.
+ACCESO A LOSA PARA CHEQUEO DE ROTOPLAS
+</t>
+  </si>
+  <si>
+    <t>C-009</t>
+  </si>
+  <si>
+    <t>3,800,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PLANTA BAJA:
+Amplia cochera techada y con portón eléctrico p/2 autos.
+Cisterna de 10,000 lts.
+1 Baño.
+Sala 
+Comedor.
+Cocina integral con barra desayunador.
+1 Recamara con closet y baño completo.
+PLANTA ALTA:
+Amplia recámara principal con balcón, baño completo con tina de hidromasaje y vestidor.
+Otras 2 recamaras con closet y baño completo c/u.
+AZOTEA:
+Área de lavado techado.
+Hermosa vista panorámica.
+Amplio ROFF GARDEN con asador.
+</t>
+  </si>
+  <si>
+    <t>C-010</t>
+  </si>
+  <si>
+    <t>1,650,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COL. MEXICO </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cochera p/1 auto con portón 
+Sala-Comedor.
+Cocina Integral.
+2 Recamara con closet.
+3 Baños completos.
+  Área de lavado. 
+.
+</t>
+  </si>
+  <si>
+    <t>C-011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CASA RESIDENCIAL </t>
+  </si>
+  <si>
+    <t>3,500,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VILLA LAS FLORES </t>
+  </si>
+  <si>
+    <t xml:space="preserve">PLANTA BAJA:
+Amplia cochera techada y con portón electrico p/2 autos.
+Pequeño espacio de jardin.
+Cisterna de 8,000 lts.
+1/2 Baño.
+Sala Concepto doble altura.
+Comedor.
+Cocina integral y con tarja moderna.
+1 Recamara con closet y baño completo.
+Pozo de luz y con lavadero.
+PLANTA ALTA:
+Amplia recamara principal con balcón, baño completo y vestidor.
+Pasillo principal con closet para blancos.
+Otras 2 recamaras con closet y baño completo c/u.
+AZOTEA:
+Área de lavado techado.
+Hermosa vista panorámica a áreas verdes.
+Amplio ROFF GARDEN.
+</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -171,6 +464,12 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <sz val="11.5"/>
+      <color rgb="FF050505"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -192,7 +491,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -205,6 +504,20 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -425,14 +738,14 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:R45"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="16" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="29.6640625" customWidth="1"/>
+    <col min="14" max="14" width="29.7109375" customWidth="1"/>
     <col min="15" max="15" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -488,7 +801,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="118.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:18" ht="118.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>23</v>
       </c>
@@ -544,7 +857,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="58.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:18" ht="58.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>28</v>
       </c>
@@ -600,207 +913,561 @@
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
-      <c r="K4" s="1"/>
-      <c r="L4" s="1"/>
-      <c r="M4" s="1"/>
-      <c r="N4" s="4"/>
-      <c r="O4" s="1"/>
-      <c r="P4" s="3"/>
-      <c r="Q4" s="1"/>
-      <c r="R4" s="1"/>
-    </row>
-    <row r="5" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1"/>
-      <c r="K5" s="1"/>
-      <c r="L5" s="1"/>
-      <c r="M5" s="1"/>
-      <c r="N5" s="4"/>
-      <c r="O5" s="1"/>
-      <c r="P5" s="3"/>
-      <c r="Q5" s="1"/>
-      <c r="R5" s="1"/>
-    </row>
-    <row r="6" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
-      <c r="K6" s="1"/>
-      <c r="L6" s="1"/>
-      <c r="M6" s="1"/>
-      <c r="N6" s="4"/>
-      <c r="O6" s="1"/>
-      <c r="P6" s="3"/>
-      <c r="Q6" s="1"/>
-      <c r="R6" s="1"/>
-    </row>
-    <row r="7" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-      <c r="J7" s="1"/>
-      <c r="K7" s="1"/>
-      <c r="L7" s="1"/>
-      <c r="M7" s="1"/>
-      <c r="N7" s="4"/>
-      <c r="O7" s="1"/>
-      <c r="P7" s="3"/>
-      <c r="Q7" s="1"/>
-      <c r="R7" s="1"/>
-    </row>
-    <row r="8" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
-      <c r="J8" s="1"/>
-      <c r="K8" s="1"/>
-      <c r="L8" s="1"/>
-      <c r="M8" s="1"/>
-      <c r="N8" s="4"/>
-      <c r="O8" s="1"/>
-      <c r="P8" s="3"/>
-      <c r="Q8" s="1"/>
-      <c r="R8" s="1"/>
-    </row>
-    <row r="9" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
-      <c r="G9" s="1"/>
-      <c r="H9" s="1"/>
-      <c r="I9" s="1"/>
-      <c r="J9" s="1"/>
-      <c r="K9" s="1"/>
-      <c r="L9" s="1"/>
-      <c r="M9" s="1"/>
-      <c r="N9" s="4"/>
-      <c r="O9" s="1"/>
-      <c r="P9" s="3"/>
-      <c r="Q9" s="1"/>
-      <c r="R9" s="1"/>
-    </row>
-    <row r="10" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="1"/>
-      <c r="I10" s="1"/>
-      <c r="J10" s="1"/>
-      <c r="K10" s="1"/>
-      <c r="L10" s="1"/>
-      <c r="M10" s="1"/>
-      <c r="N10" s="4"/>
-      <c r="O10" s="1"/>
-      <c r="P10" s="3"/>
-      <c r="Q10" s="1"/>
-      <c r="R10" s="1"/>
-    </row>
-    <row r="11" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
-      <c r="G11" s="1"/>
-      <c r="H11" s="1"/>
-      <c r="I11" s="1"/>
-      <c r="J11" s="1"/>
-      <c r="K11" s="1"/>
-      <c r="L11" s="1"/>
-      <c r="M11" s="1"/>
-      <c r="N11" s="4"/>
-      <c r="O11" s="1"/>
-      <c r="P11" s="3"/>
-      <c r="Q11" s="1"/>
-      <c r="R11" s="1"/>
-    </row>
-    <row r="12" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
-      <c r="G12" s="1"/>
-      <c r="H12" s="1"/>
-      <c r="I12" s="1"/>
-      <c r="J12" s="1"/>
-      <c r="K12" s="1"/>
-      <c r="L12" s="1"/>
-      <c r="M12" s="1"/>
-      <c r="N12" s="4"/>
-      <c r="O12" s="1"/>
-      <c r="P12" s="3"/>
-      <c r="Q12" s="1"/>
-      <c r="R12" s="1"/>
-    </row>
-    <row r="13" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="1"/>
-      <c r="H13" s="1"/>
-      <c r="I13" s="1"/>
-      <c r="J13" s="1"/>
-      <c r="K13" s="1"/>
-      <c r="L13" s="1"/>
-      <c r="M13" s="1"/>
-      <c r="N13" s="4"/>
-      <c r="O13" s="1"/>
-      <c r="P13" s="3"/>
-      <c r="Q13" s="1"/>
-      <c r="R13" s="1"/>
-    </row>
-    <row r="14" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="J4" s="7">
+        <v>0</v>
+      </c>
+      <c r="K4" s="7">
+        <v>0</v>
+      </c>
+      <c r="L4" s="7">
+        <v>0</v>
+      </c>
+      <c r="M4" s="7">
+        <v>0</v>
+      </c>
+      <c r="N4" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="O4" s="9">
+        <v>2281470383</v>
+      </c>
+      <c r="P4" s="8">
+        <v>46120</v>
+      </c>
+      <c r="Q4" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="R4" s="7" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="I5" s="7">
+        <v>105</v>
+      </c>
+      <c r="J5" s="7">
+        <v>158</v>
+      </c>
+      <c r="K5" s="7">
+        <v>3</v>
+      </c>
+      <c r="L5" s="7">
+        <v>3</v>
+      </c>
+      <c r="M5" s="7">
+        <v>1</v>
+      </c>
+      <c r="N5" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="O5" s="9">
+        <v>2281470383</v>
+      </c>
+      <c r="P5" s="8">
+        <v>46120</v>
+      </c>
+      <c r="Q5" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="R5" s="7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="I6" s="7"/>
+      <c r="J6" s="7"/>
+      <c r="K6" s="7">
+        <v>2</v>
+      </c>
+      <c r="L6" s="7">
+        <v>1</v>
+      </c>
+      <c r="M6" s="7">
+        <v>1</v>
+      </c>
+      <c r="N6" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="O6" s="9">
+        <v>2281470383</v>
+      </c>
+      <c r="P6" s="8">
+        <v>46120</v>
+      </c>
+      <c r="Q6" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="R6" s="7" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="I7" s="7">
+        <v>143</v>
+      </c>
+      <c r="J7" s="7">
+        <v>350</v>
+      </c>
+      <c r="K7" s="7">
+        <v>4</v>
+      </c>
+      <c r="L7" s="7">
+        <v>3</v>
+      </c>
+      <c r="M7" s="7">
+        <v>3</v>
+      </c>
+      <c r="N7" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="O7" s="9">
+        <v>2281470383</v>
+      </c>
+      <c r="P7" s="8">
+        <v>46120</v>
+      </c>
+      <c r="Q7" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="R7" s="7" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="I8" s="7">
+        <v>105</v>
+      </c>
+      <c r="J8" s="7">
+        <v>146</v>
+      </c>
+      <c r="K8" s="7">
+        <v>3</v>
+      </c>
+      <c r="L8" s="7">
+        <v>4</v>
+      </c>
+      <c r="M8" s="7">
+        <v>1</v>
+      </c>
+      <c r="N8" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="O8" s="9">
+        <v>2281470383</v>
+      </c>
+      <c r="P8" s="8">
+        <v>46120</v>
+      </c>
+      <c r="Q8" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="R8" s="7" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="I9" s="7">
+        <v>120</v>
+      </c>
+      <c r="J9" s="7">
+        <v>150</v>
+      </c>
+      <c r="K9" s="7">
+        <v>3</v>
+      </c>
+      <c r="L9" s="7">
+        <v>4</v>
+      </c>
+      <c r="M9" s="7">
+        <v>2</v>
+      </c>
+      <c r="N9" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="O9" s="9">
+        <v>2281470383</v>
+      </c>
+      <c r="P9" s="8">
+        <v>46120</v>
+      </c>
+      <c r="Q9" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="R9" s="7" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="I10" s="7">
+        <v>105</v>
+      </c>
+      <c r="J10" s="7">
+        <v>198</v>
+      </c>
+      <c r="K10" s="7">
+        <v>3</v>
+      </c>
+      <c r="L10" s="7">
+        <v>4</v>
+      </c>
+      <c r="M10" s="7">
+        <v>2</v>
+      </c>
+      <c r="N10" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="O10" s="9">
+        <v>2281470383</v>
+      </c>
+      <c r="P10" s="8">
+        <v>46120</v>
+      </c>
+      <c r="Q10" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="R10" s="7" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="G11" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="I11" s="7">
+        <v>171</v>
+      </c>
+      <c r="J11" s="7">
+        <v>220</v>
+      </c>
+      <c r="K11" s="7">
+        <v>4</v>
+      </c>
+      <c r="L11" s="7">
+        <v>4</v>
+      </c>
+      <c r="M11" s="7">
+        <v>2</v>
+      </c>
+      <c r="N11" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="O11" s="9">
+        <v>2281470383</v>
+      </c>
+      <c r="P11" s="8">
+        <v>46120</v>
+      </c>
+      <c r="Q11" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="R11" s="7" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="I12" s="7">
+        <v>126</v>
+      </c>
+      <c r="J12" s="7"/>
+      <c r="K12" s="7">
+        <v>2</v>
+      </c>
+      <c r="L12" s="7">
+        <v>1</v>
+      </c>
+      <c r="M12" s="7">
+        <v>1</v>
+      </c>
+      <c r="N12" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="O12" s="7">
+        <v>2281852255</v>
+      </c>
+      <c r="P12" s="8">
+        <v>46120</v>
+      </c>
+      <c r="Q12" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="R12" s="7" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="I13" s="7">
+        <v>120</v>
+      </c>
+      <c r="J13" s="7">
+        <v>230</v>
+      </c>
+      <c r="K13" s="7">
+        <v>4</v>
+      </c>
+      <c r="L13" s="7">
+        <v>5</v>
+      </c>
+      <c r="M13" s="7">
+        <v>2</v>
+      </c>
+      <c r="N13" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="O13" s="7">
+        <v>2281852255</v>
+      </c>
+      <c r="P13" s="8">
+        <v>46120</v>
+      </c>
+      <c r="Q13" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="R13" s="7" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -820,7 +1487,7 @@
       <c r="Q14" s="1"/>
       <c r="R14" s="1"/>
     </row>
-    <row r="15" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -840,7 +1507,7 @@
       <c r="Q15" s="1"/>
       <c r="R15" s="1"/>
     </row>
-    <row r="16" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
@@ -860,7 +1527,7 @@
       <c r="Q16" s="1"/>
       <c r="R16" s="1"/>
     </row>
-    <row r="17" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
@@ -880,7 +1547,7 @@
       <c r="Q17" s="1"/>
       <c r="R17" s="1"/>
     </row>
-    <row r="18" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -900,7 +1567,7 @@
       <c r="Q18" s="1"/>
       <c r="R18" s="1"/>
     </row>
-    <row r="19" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -920,7 +1587,7 @@
       <c r="Q19" s="1"/>
       <c r="R19" s="1"/>
     </row>
-    <row r="20" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
@@ -940,7 +1607,7 @@
       <c r="Q20" s="1"/>
       <c r="R20" s="1"/>
     </row>
-    <row r="21" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
@@ -960,7 +1627,7 @@
       <c r="Q21" s="1"/>
       <c r="R21" s="1"/>
     </row>
-    <row r="22" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
@@ -980,7 +1647,7 @@
       <c r="Q22" s="1"/>
       <c r="R22" s="1"/>
     </row>
-    <row r="23" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="23" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
@@ -1000,7 +1667,7 @@
       <c r="Q23" s="2"/>
       <c r="R23" s="2"/>
     </row>
-    <row r="24" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
@@ -1020,7 +1687,7 @@
       <c r="Q24" s="1"/>
       <c r="R24" s="1"/>
     </row>
-    <row r="25" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="25" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
@@ -1040,7 +1707,7 @@
       <c r="Q25" s="1"/>
       <c r="R25" s="1"/>
     </row>
-    <row r="26" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -1060,7 +1727,7 @@
       <c r="Q26" s="1"/>
       <c r="R26" s="1"/>
     </row>
-    <row r="27" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="27" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
@@ -1080,7 +1747,7 @@
       <c r="Q27" s="1"/>
       <c r="R27" s="1"/>
     </row>
-    <row r="28" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="28" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -1100,7 +1767,7 @@
       <c r="Q28" s="1"/>
       <c r="R28" s="1"/>
     </row>
-    <row r="29" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="29" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -1120,7 +1787,7 @@
       <c r="Q29" s="1"/>
       <c r="R29" s="1"/>
     </row>
-    <row r="30" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="30" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
@@ -1140,7 +1807,7 @@
       <c r="Q30" s="1"/>
       <c r="R30" s="1"/>
     </row>
-    <row r="31" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="31" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
@@ -1160,7 +1827,7 @@
       <c r="Q31" s="1"/>
       <c r="R31" s="1"/>
     </row>
-    <row r="32" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="32" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
@@ -1180,7 +1847,7 @@
       <c r="Q32" s="1"/>
       <c r="R32" s="1"/>
     </row>
-    <row r="33" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="33" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
@@ -1200,7 +1867,7 @@
       <c r="Q33" s="1"/>
       <c r="R33" s="1"/>
     </row>
-    <row r="34" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="34" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
@@ -1220,7 +1887,7 @@
       <c r="Q34" s="1"/>
       <c r="R34" s="1"/>
     </row>
-    <row r="35" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="35" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
       <c r="C35" s="1"/>
@@ -1240,7 +1907,7 @@
       <c r="Q35" s="1"/>
       <c r="R35" s="1"/>
     </row>
-    <row r="36" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="36" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="1"/>
       <c r="B36" s="1"/>
       <c r="C36" s="1"/>
@@ -1260,7 +1927,7 @@
       <c r="Q36" s="1"/>
       <c r="R36" s="1"/>
     </row>
-    <row r="37" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="37" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="1"/>
       <c r="B37" s="1"/>
       <c r="C37" s="1"/>
@@ -1280,7 +1947,7 @@
       <c r="Q37" s="1"/>
       <c r="R37" s="1"/>
     </row>
-    <row r="38" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="38" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="1"/>
       <c r="B38" s="1"/>
       <c r="C38" s="1"/>
@@ -1300,7 +1967,7 @@
       <c r="Q38" s="1"/>
       <c r="R38" s="1"/>
     </row>
-    <row r="39" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="39" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
       <c r="C39" s="1"/>
@@ -1320,7 +1987,7 @@
       <c r="Q39" s="1"/>
       <c r="R39" s="1"/>
     </row>
-    <row r="40" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="40" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="1"/>
       <c r="B40" s="1"/>
       <c r="C40" s="1"/>
@@ -1340,7 +2007,7 @@
       <c r="Q40" s="1"/>
       <c r="R40" s="1"/>
     </row>
-    <row r="41" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="41" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
       <c r="C41" s="1"/>
@@ -1360,7 +2027,7 @@
       <c r="Q41" s="1"/>
       <c r="R41" s="1"/>
     </row>
-    <row r="42" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="42" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="1"/>
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
@@ -1380,7 +2047,7 @@
       <c r="Q42" s="1"/>
       <c r="R42" s="1"/>
     </row>
-    <row r="43" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="43" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
@@ -1400,7 +2067,7 @@
       <c r="Q43" s="1"/>
       <c r="R43" s="1"/>
     </row>
-    <row r="44" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="44" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
       <c r="C44" s="1"/>
@@ -1420,7 +2087,7 @@
       <c r="Q44" s="1"/>
       <c r="R44" s="1"/>
     </row>
-    <row r="45" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="45" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
       <c r="C45" s="1"/>

</xml_diff>

<commit_message>
Update: Agregadas nuevas propiedades y fotos
</commit_message>
<xml_diff>
--- a/casas.xlsx
+++ b/casas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hans_\OneDrive\Escritorio\Projectos\Real State\gestioninmobiliargalindo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47D3990E-72F2-46CA-8BAD-C7684670B99B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48071387-C013-41F3-B92D-8D08005DD4D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="28800" windowHeight="15285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38400" yWindow="750" windowWidth="28800" windowHeight="15285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template Excel para Script Pyth" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="72">
   <si>
     <t>id</t>
   </si>
@@ -148,16 +148,10 @@
     <t xml:space="preserve">VENTA </t>
   </si>
   <si>
-    <t>1,050,000</t>
-  </si>
-  <si>
     <t xml:space="preserve">EL HAYA </t>
   </si>
   <si>
     <t>Xalapa</t>
-  </si>
-  <si>
-    <t>330.3</t>
   </si>
   <si>
     <t xml:space="preserve">UBICADO EN EL HAYA 
@@ -174,9 +168,6 @@
   </si>
   <si>
     <t xml:space="preserve">CASA HABITACION </t>
-  </si>
-  <si>
-    <t>2,100,000</t>
   </si>
   <si>
     <t xml:space="preserve">JARDINES </t>
@@ -219,9 +210,6 @@
     <t>DEPARTAMENTO</t>
   </si>
   <si>
-    <t>1,550,000</t>
-  </si>
-  <si>
     <t xml:space="preserve">DEPARTAMENTOS  UBICADOS AUN COSTADO DE PLAZA CRISTAL 
                                    $ 1,550,000
 Cajón de estacionamiento p/1 auto (la cochera es techada y con portón eléctrico).
@@ -236,9 +224,6 @@
   </si>
   <si>
     <t>C-005</t>
-  </si>
-  <si>
-    <t>3,000,000</t>
   </si>
   <si>
     <t xml:space="preserve">TRANCAS </t>
@@ -276,9 +261,6 @@
     <t xml:space="preserve">RESIDENCIAL LIRIOS </t>
   </si>
   <si>
-    <t>2,500,000</t>
-  </si>
-  <si>
     <t xml:space="preserve">COATEPEC </t>
   </si>
   <si>
@@ -306,9 +288,6 @@
     <t>C-007</t>
   </si>
   <si>
-    <t>2,240,000</t>
-  </si>
-  <si>
     <t xml:space="preserve">PLANTA BAJA:
 Amplia cochera p/2 autos.
 1 Baño de visitas.
@@ -328,9 +307,6 @@
   </si>
   <si>
     <t>CASARESIDENCIAL</t>
-  </si>
-  <si>
-    <t>3,190,000</t>
   </si>
   <si>
     <t>MORADA DEL QUETZAL</t>
@@ -359,9 +335,6 @@
     <t>C-009</t>
   </si>
   <si>
-    <t>3,800,000</t>
-  </si>
-  <si>
     <t xml:space="preserve">PLANTA BAJA:
 Amplia cochera techada y con portón eléctrico p/2 autos.
 Cisterna de 10,000 lts.
@@ -383,9 +356,6 @@
     <t>C-010</t>
   </si>
   <si>
-    <t>1,650,000</t>
-  </si>
-  <si>
     <t xml:space="preserve">COL. MEXICO </t>
   </si>
   <si>
@@ -403,9 +373,6 @@
   </si>
   <si>
     <t xml:space="preserve">CASA RESIDENCIAL </t>
-  </si>
-  <si>
-    <t>3,500,000</t>
   </si>
   <si>
     <t xml:space="preserve">VILLA LAS FLORES </t>
@@ -491,7 +458,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -505,20 +472,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -914,557 +875,557 @@
       </c>
     </row>
     <row r="4" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="10">
+        <v>1050000</v>
+      </c>
+      <c r="G4" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="H4" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="I4" s="9">
+        <v>330.3</v>
+      </c>
+      <c r="J4" s="1">
+        <v>0</v>
+      </c>
+      <c r="K4" s="1">
+        <v>0</v>
+      </c>
+      <c r="L4" s="1">
+        <v>0</v>
+      </c>
+      <c r="M4" s="1">
+        <v>0</v>
+      </c>
+      <c r="N4" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="I4" s="7" t="s">
+      <c r="O4" s="7">
+        <v>2281470383</v>
+      </c>
+      <c r="P4" s="3">
+        <v>46120</v>
+      </c>
+      <c r="Q4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="R4" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="J4" s="7">
-        <v>0</v>
-      </c>
-      <c r="K4" s="7">
-        <v>0</v>
-      </c>
-      <c r="L4" s="7">
-        <v>0</v>
-      </c>
-      <c r="M4" s="7">
-        <v>0</v>
-      </c>
-      <c r="N4" s="10" t="s">
+      <c r="B5" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="O4" s="9">
+      <c r="C5" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F5" s="10">
+        <v>2100000</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="I5" s="1">
+        <v>105</v>
+      </c>
+      <c r="J5" s="1">
+        <v>158</v>
+      </c>
+      <c r="K5" s="1">
+        <v>3</v>
+      </c>
+      <c r="L5" s="1">
+        <v>3</v>
+      </c>
+      <c r="M5" s="1">
+        <v>1</v>
+      </c>
+      <c r="N5" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="O5" s="7">
         <v>2281470383</v>
       </c>
-      <c r="P4" s="8">
+      <c r="P5" s="3">
         <v>46120</v>
       </c>
-      <c r="Q4" s="7" t="s">
+      <c r="Q5" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="R4" s="7" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="7" t="s">
+      <c r="R5" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F6" s="10">
+        <v>1550000</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1">
+        <v>2</v>
+      </c>
+      <c r="L6" s="1">
+        <v>1</v>
+      </c>
+      <c r="M6" s="1">
+        <v>1</v>
+      </c>
+      <c r="N6" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="O6" s="7">
+        <v>2281470383</v>
+      </c>
+      <c r="P6" s="3">
+        <v>46120</v>
+      </c>
+      <c r="Q6" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="R6" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="D5" s="7" t="s">
+      <c r="D7" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E5" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="I5" s="7">
+      <c r="E7" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F7" s="10">
+        <v>3000000</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="I7" s="1">
+        <v>143</v>
+      </c>
+      <c r="J7" s="1">
+        <v>350</v>
+      </c>
+      <c r="K7" s="1">
+        <v>4</v>
+      </c>
+      <c r="L7" s="1">
+        <v>3</v>
+      </c>
+      <c r="M7" s="1">
+        <v>3</v>
+      </c>
+      <c r="N7" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="O7" s="7">
+        <v>2281470383</v>
+      </c>
+      <c r="P7" s="3">
+        <v>46120</v>
+      </c>
+      <c r="Q7" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="R7" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F8" s="10">
+        <v>2500000</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="I8" s="1">
         <v>105</v>
       </c>
-      <c r="J5" s="7">
-        <v>158</v>
-      </c>
-      <c r="K5" s="7">
+      <c r="J8" s="1">
+        <v>146</v>
+      </c>
+      <c r="K8" s="1">
         <v>3</v>
       </c>
-      <c r="L5" s="7">
+      <c r="L8" s="1">
+        <v>4</v>
+      </c>
+      <c r="M8" s="1">
+        <v>1</v>
+      </c>
+      <c r="N8" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="O8" s="7">
+        <v>2281470383</v>
+      </c>
+      <c r="P8" s="3">
+        <v>46120</v>
+      </c>
+      <c r="Q8" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="R8" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F9" s="10">
+        <v>2240000</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="I9" s="1">
+        <v>120</v>
+      </c>
+      <c r="J9" s="1">
+        <v>150</v>
+      </c>
+      <c r="K9" s="1">
         <v>3</v>
       </c>
-      <c r="M5" s="7">
+      <c r="L9" s="1">
+        <v>4</v>
+      </c>
+      <c r="M9" s="1">
+        <v>2</v>
+      </c>
+      <c r="N9" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="O9" s="7">
+        <v>2281470383</v>
+      </c>
+      <c r="P9" s="3">
+        <v>46120</v>
+      </c>
+      <c r="Q9" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="R9" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F10" s="10">
+        <v>3190000</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="I10" s="1">
+        <v>105</v>
+      </c>
+      <c r="J10" s="1">
+        <v>198</v>
+      </c>
+      <c r="K10" s="1">
+        <v>3</v>
+      </c>
+      <c r="L10" s="1">
+        <v>4</v>
+      </c>
+      <c r="M10" s="1">
+        <v>2</v>
+      </c>
+      <c r="N10" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="O10" s="7">
+        <v>2281470383</v>
+      </c>
+      <c r="P10" s="3">
+        <v>46120</v>
+      </c>
+      <c r="Q10" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="R10" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F11" s="10">
+        <v>3800000</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="I11" s="1">
+        <v>171</v>
+      </c>
+      <c r="J11" s="1">
+        <v>220</v>
+      </c>
+      <c r="K11" s="1">
+        <v>4</v>
+      </c>
+      <c r="L11" s="1">
+        <v>4</v>
+      </c>
+      <c r="M11" s="1">
+        <v>2</v>
+      </c>
+      <c r="N11" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="O11" s="7">
+        <v>2281470383</v>
+      </c>
+      <c r="P11" s="3">
+        <v>46120</v>
+      </c>
+      <c r="Q11" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="R11" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F12" s="10">
+        <v>1650000</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="I12" s="1">
+        <v>126</v>
+      </c>
+      <c r="J12" s="1"/>
+      <c r="K12" s="1">
+        <v>2</v>
+      </c>
+      <c r="L12" s="1">
         <v>1</v>
       </c>
-      <c r="N5" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="O5" s="9">
-        <v>2281470383</v>
-      </c>
-      <c r="P5" s="8">
+      <c r="M12" s="1">
+        <v>1</v>
+      </c>
+      <c r="N12" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="O12" s="1">
+        <v>2281852255</v>
+      </c>
+      <c r="P12" s="3">
         <v>46120</v>
       </c>
-      <c r="Q5" s="7" t="s">
+      <c r="Q12" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="R5" s="7" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="E6" s="7" t="s">
+      <c r="R12" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F13" s="10">
+        <v>3500000</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="H13" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="F6" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="I6" s="7"/>
-      <c r="J6" s="7"/>
-      <c r="K6" s="7">
+      <c r="I13" s="1">
+        <v>120</v>
+      </c>
+      <c r="J13" s="1">
+        <v>230</v>
+      </c>
+      <c r="K13" s="1">
+        <v>4</v>
+      </c>
+      <c r="L13" s="1">
+        <v>5</v>
+      </c>
+      <c r="M13" s="1">
         <v>2</v>
       </c>
-      <c r="L6" s="7">
-        <v>1</v>
-      </c>
-      <c r="M6" s="7">
-        <v>1</v>
-      </c>
-      <c r="N6" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="O6" s="9">
-        <v>2281470383</v>
-      </c>
-      <c r="P6" s="8">
+      <c r="N13" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="O13" s="1">
+        <v>2281852255</v>
+      </c>
+      <c r="P13" s="3">
         <v>46120</v>
       </c>
-      <c r="Q6" s="7" t="s">
+      <c r="Q13" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="R6" s="7" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="7" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="I7" s="7">
-        <v>143</v>
-      </c>
-      <c r="J7" s="7">
-        <v>350</v>
-      </c>
-      <c r="K7" s="7">
-        <v>4</v>
-      </c>
-      <c r="L7" s="7">
-        <v>3</v>
-      </c>
-      <c r="M7" s="7">
-        <v>3</v>
-      </c>
-      <c r="N7" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="O7" s="9">
-        <v>2281470383</v>
-      </c>
-      <c r="P7" s="8">
-        <v>46120</v>
-      </c>
-      <c r="Q7" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="R7" s="7" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="8" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="H8" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="I8" s="7">
-        <v>105</v>
-      </c>
-      <c r="J8" s="7">
-        <v>146</v>
-      </c>
-      <c r="K8" s="7">
-        <v>3</v>
-      </c>
-      <c r="L8" s="7">
-        <v>4</v>
-      </c>
-      <c r="M8" s="7">
-        <v>1</v>
-      </c>
-      <c r="N8" s="11" t="s">
-        <v>62</v>
-      </c>
-      <c r="O8" s="9">
-        <v>2281470383</v>
-      </c>
-      <c r="P8" s="8">
-        <v>46120</v>
-      </c>
-      <c r="Q8" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="R8" s="7" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="9" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="G9" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="H9" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="I9" s="7">
-        <v>120</v>
-      </c>
-      <c r="J9" s="7">
-        <v>150</v>
-      </c>
-      <c r="K9" s="7">
-        <v>3</v>
-      </c>
-      <c r="L9" s="7">
-        <v>4</v>
-      </c>
-      <c r="M9" s="7">
-        <v>2</v>
-      </c>
-      <c r="N9" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="O9" s="9">
-        <v>2281470383</v>
-      </c>
-      <c r="P9" s="8">
-        <v>46120</v>
-      </c>
-      <c r="Q9" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="R9" s="7" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="10" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="F10" s="7" t="s">
+      <c r="R13" s="1" t="s">
         <v>68</v>
-      </c>
-      <c r="G10" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H10" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="I10" s="7">
-        <v>105</v>
-      </c>
-      <c r="J10" s="7">
-        <v>198</v>
-      </c>
-      <c r="K10" s="7">
-        <v>3</v>
-      </c>
-      <c r="L10" s="7">
-        <v>4</v>
-      </c>
-      <c r="M10" s="7">
-        <v>2</v>
-      </c>
-      <c r="N10" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="O10" s="9">
-        <v>2281470383</v>
-      </c>
-      <c r="P10" s="8">
-        <v>46120</v>
-      </c>
-      <c r="Q10" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="R10" s="7" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="11" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="E11" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="F11" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="G11" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="H11" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="I11" s="7">
-        <v>171</v>
-      </c>
-      <c r="J11" s="7">
-        <v>220</v>
-      </c>
-      <c r="K11" s="7">
-        <v>4</v>
-      </c>
-      <c r="L11" s="7">
-        <v>4</v>
-      </c>
-      <c r="M11" s="7">
-        <v>2</v>
-      </c>
-      <c r="N11" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="O11" s="9">
-        <v>2281470383</v>
-      </c>
-      <c r="P11" s="8">
-        <v>46120</v>
-      </c>
-      <c r="Q11" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="R11" s="7" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="12" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="G12" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="H12" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="I12" s="7">
-        <v>126</v>
-      </c>
-      <c r="J12" s="7"/>
-      <c r="K12" s="7">
-        <v>2</v>
-      </c>
-      <c r="L12" s="7">
-        <v>1</v>
-      </c>
-      <c r="M12" s="7">
-        <v>1</v>
-      </c>
-      <c r="N12" s="12" t="s">
-        <v>77</v>
-      </c>
-      <c r="O12" s="7">
-        <v>2281852255</v>
-      </c>
-      <c r="P12" s="8">
-        <v>46120</v>
-      </c>
-      <c r="Q12" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="R12" s="7" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="13" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="E13" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="G13" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="H13" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="I13" s="7">
-        <v>120</v>
-      </c>
-      <c r="J13" s="7">
-        <v>230</v>
-      </c>
-      <c r="K13" s="7">
-        <v>4</v>
-      </c>
-      <c r="L13" s="7">
-        <v>5</v>
-      </c>
-      <c r="M13" s="7">
-        <v>2</v>
-      </c>
-      <c r="N13" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="O13" s="7">
-        <v>2281852255</v>
-      </c>
-      <c r="P13" s="8">
-        <v>46120</v>
-      </c>
-      <c r="Q13" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="R13" s="7" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="14" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Unificación de estructura, JSON plano y nombres de propiedades reales
</commit_message>
<xml_diff>
--- a/casas.xlsx
+++ b/casas.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hans_\OneDrive\Escritorio\Projectos\Real State\gestioninmobiliargalindo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hans_\OneDrive\Escritorio\Projectos\Desarrollos FEr\gestioninmobiliargalindo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48071387-C013-41F3-B92D-8D08005DD4D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D93D345-24AA-4CE6-ADC3-D2FC57C89A31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38400" yWindow="750" windowWidth="28800" windowHeight="15285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="44130" yWindow="3870" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template Excel para Script Pyth" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="75">
   <si>
     <t>id</t>
   </si>
@@ -74,9 +74,6 @@
   </si>
   <si>
     <t>estatus</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campestre </t>
   </si>
   <si>
     <t xml:space="preserve">casa </t>
@@ -127,9 +124,6 @@
 </t>
   </si>
   <si>
-    <t>Residencial</t>
-  </si>
-  <si>
     <t>Venta</t>
   </si>
   <si>
@@ -165,9 +159,6 @@
   </si>
   <si>
     <t xml:space="preserve">CASA </t>
-  </si>
-  <si>
-    <t xml:space="preserve">CASA HABITACION </t>
   </si>
   <si>
     <t xml:space="preserve">JARDINES </t>
@@ -196,12 +187,6 @@
   </si>
   <si>
     <t>D-001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DEPRTANTO </t>
-  </si>
-  <si>
-    <t xml:space="preserve">DEPRTAMENTO ZONA JARDINES </t>
   </si>
   <si>
     <t>VENTA</t>
@@ -258,9 +243,6 @@
     <t>C-006</t>
   </si>
   <si>
-    <t xml:space="preserve">RESIDENCIAL LIRIOS </t>
-  </si>
-  <si>
     <t xml:space="preserve">COATEPEC </t>
   </si>
   <si>
@@ -304,9 +286,6 @@
   </si>
   <si>
     <t>C-008</t>
-  </si>
-  <si>
-    <t>CASARESIDENCIAL</t>
   </si>
   <si>
     <t>MORADA DEL QUETZAL</t>
@@ -370,9 +349,6 @@
   </si>
   <si>
     <t>C-011</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CASA RESIDENCIAL </t>
   </si>
   <si>
     <t xml:space="preserve">VILLA LAS FLORES </t>
@@ -397,6 +373,39 @@
 Hermosa vista panorámica a áreas verdes.
 Amplio ROFF GARDEN.
 </t>
+  </si>
+  <si>
+    <t>CAMPESTRE</t>
+  </si>
+  <si>
+    <t>RESIDENCIAL</t>
+  </si>
+  <si>
+    <t>TERRENO</t>
+  </si>
+  <si>
+    <t>CASA JARDINES</t>
+  </si>
+  <si>
+    <t>CASA TRANCAS</t>
+  </si>
+  <si>
+    <t>CASA COATEPEC</t>
+  </si>
+  <si>
+    <t>CASA TRANCAS II</t>
+  </si>
+  <si>
+    <t>CASA MORADA DEL QUETZAL</t>
+  </si>
+  <si>
+    <t>CASA TRANCAS III</t>
+  </si>
+  <si>
+    <t>CASA COL. MEXICO</t>
+  </si>
+  <si>
+    <t>CASA VILLA LAS FLORES</t>
   </si>
 </sst>
 </file>
@@ -446,12 +455,27 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -478,8 +502,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -706,7 +732,7 @@
     <col min="15" max="15" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -762,30 +788,30 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="118.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:18" ht="118.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>18</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>19</v>
       </c>
       <c r="F2" s="1">
         <v>8500000</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I2" s="1">
         <v>3.7130000000000001</v>
@@ -803,7 +829,7 @@
         <v>7</v>
       </c>
       <c r="N2" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="O2" s="6">
         <v>2281852255</v>
@@ -812,36 +838,36 @@
         <v>46115</v>
       </c>
       <c r="Q2" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="R2" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18" ht="58.5" customHeight="1" x14ac:dyDescent="0.2">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" ht="58.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B3" s="1" t="s">
         <v>26</v>
       </c>
+      <c r="B3" s="10" t="s">
+        <v>65</v>
+      </c>
       <c r="C3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>18</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>19</v>
       </c>
       <c r="F3" s="1">
         <v>4250000</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I3" s="1">
         <v>143</v>
@@ -859,7 +885,7 @@
         <v>2</v>
       </c>
       <c r="N3" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="O3" s="6">
         <v>2281852255</v>
@@ -868,38 +894,38 @@
         <v>46115</v>
       </c>
       <c r="Q3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="R3" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="R3" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="4" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B4" s="1" t="s">
+      <c r="F4" s="9">
+        <v>1050000</v>
+      </c>
+      <c r="G4" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="D4" s="1" t="s">
+      <c r="H4" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="F4" s="10">
-        <v>1050000</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="I4" s="9">
+      <c r="I4" s="1">
         <v>330.3</v>
       </c>
       <c r="J4" s="1">
@@ -915,7 +941,7 @@
         <v>0</v>
       </c>
       <c r="N4" s="8" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="O4" s="7">
         <v>2281470383</v>
@@ -924,36 +950,36 @@
         <v>46120</v>
       </c>
       <c r="Q4" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="R4" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="5" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="1" t="s">
+      <c r="E5" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="F5" s="9">
+        <v>2100000</v>
+      </c>
+      <c r="G5" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>37</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F5" s="10">
-        <v>2100000</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>40</v>
       </c>
       <c r="I5" s="1">
         <v>105</v>
@@ -971,7 +997,7 @@
         <v>1</v>
       </c>
       <c r="N5" s="8" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="O5" s="7">
         <v>2281470383</v>
@@ -980,36 +1006,36 @@
         <v>46120</v>
       </c>
       <c r="Q5" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="R5" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F6" s="9">
+        <v>1550000</v>
+      </c>
+      <c r="G6" s="1" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="6" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="F6" s="10">
-        <v>1550000</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>39</v>
-      </c>
       <c r="H6" s="1" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
@@ -1023,7 +1049,7 @@
         <v>1</v>
       </c>
       <c r="N6" s="8" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="O6" s="7">
         <v>2281470383</v>
@@ -1032,36 +1058,36 @@
         <v>46120</v>
       </c>
       <c r="Q6" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="R6" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="7" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>37</v>
+        <v>43</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>68</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F7" s="10">
+        <v>35</v>
+      </c>
+      <c r="F7" s="9">
         <v>3000000</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="I7" s="1">
         <v>143</v>
@@ -1079,7 +1105,7 @@
         <v>3</v>
       </c>
       <c r="N7" s="8" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="O7" s="7">
         <v>2281470383</v>
@@ -1088,36 +1114,36 @@
         <v>46120</v>
       </c>
       <c r="Q7" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="R7" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="F8" s="9">
+        <v>2500000</v>
+      </c>
+      <c r="G8" s="1" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="8" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F8" s="10">
-        <v>2500000</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>54</v>
-      </c>
       <c r="H8" s="1" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="I8" s="1">
         <v>105</v>
@@ -1135,7 +1161,7 @@
         <v>1</v>
       </c>
       <c r="N8" s="6" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="O8" s="7">
         <v>2281470383</v>
@@ -1144,36 +1170,36 @@
         <v>46120</v>
       </c>
       <c r="Q8" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="R8" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="9" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>37</v>
+        <v>51</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>70</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F9" s="10">
+        <v>35</v>
+      </c>
+      <c r="F9" s="9">
         <v>2240000</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="I9" s="1">
         <v>120</v>
@@ -1191,7 +1217,7 @@
         <v>2</v>
       </c>
       <c r="N9" s="6" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="O9" s="7">
         <v>2281470383</v>
@@ -1200,36 +1226,36 @@
         <v>46120</v>
       </c>
       <c r="Q9" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="R9" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="10" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>37</v>
+        <v>53</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>71</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F10" s="10">
+        <v>35</v>
+      </c>
+      <c r="F10" s="9">
         <v>3190000</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="I10" s="1">
         <v>105</v>
@@ -1247,7 +1273,7 @@
         <v>2</v>
       </c>
       <c r="N10" s="6" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="O10" s="7">
         <v>2281470383</v>
@@ -1256,36 +1282,36 @@
         <v>46120</v>
       </c>
       <c r="Q10" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="R10" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="11" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>37</v>
+        <v>56</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>72</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>38</v>
+        <v>56</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F11" s="10">
+        <v>35</v>
+      </c>
+      <c r="F11" s="9">
         <v>3800000</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="I11" s="1">
         <v>171</v>
@@ -1303,7 +1329,7 @@
         <v>2</v>
       </c>
       <c r="N11" s="5" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="O11" s="7">
         <v>2281470383</v>
@@ -1312,36 +1338,36 @@
         <v>46120</v>
       </c>
       <c r="Q11" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="R11" s="1" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="12" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>37</v>
+        <v>58</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>73</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>38</v>
+        <v>58</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F12" s="10">
+        <v>35</v>
+      </c>
+      <c r="F12" s="9">
         <v>1650000</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="I12" s="1">
         <v>126</v>
@@ -1357,7 +1383,7 @@
         <v>1</v>
       </c>
       <c r="N12" s="5" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="O12" s="1">
         <v>2281852255</v>
@@ -1366,36 +1392,36 @@
         <v>46120</v>
       </c>
       <c r="Q12" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="R12" s="1" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="13" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>37</v>
+        <v>61</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>74</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F13" s="10">
+        <v>35</v>
+      </c>
+      <c r="F13" s="9">
         <v>3500000</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="I13" s="1">
         <v>120</v>
@@ -1413,7 +1439,7 @@
         <v>2</v>
       </c>
       <c r="N13" s="5" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="O13" s="1">
         <v>2281852255</v>
@@ -1422,10 +1448,10 @@
         <v>46120</v>
       </c>
       <c r="Q13" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="R13" s="1" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
     </row>
     <row r="14" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>